<commit_message>
Error checks for Timeslice sheets working
</commit_message>
<xml_diff>
--- a/GENeSYS-MOD_User_Input_Settings_v03_phe_06-09-2023.xlsx
+++ b/GENeSYS-MOD_User_Input_Settings_v03_phe_06-09-2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dozeumhep\Documents\git\GENeSYS-MOD_GroupRepo\GENeSYS-MOD_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E159838-42F4-4374-AE33-1D4B85A761EA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{870C1A07-6CC8-4107-B661-2B817B103036}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0B764928-35F8-4A30-ADCD-C0369050184D}"/>
   </bookViews>
@@ -1187,12 +1187,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A667788-FC3C-4C43-9E46-ED47A2AEE749}">
   <dimension ref="A1:C40"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>260</v>
       </c>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1209,7 +1209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1217,7 +1217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1225,7 +1225,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1233,7 +1233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -1241,7 +1241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -1249,7 +1249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1265,7 +1265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1273,7 +1273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -1281,7 +1281,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -1289,7 +1289,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -1297,7 +1297,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -1313,7 +1313,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -1321,7 +1321,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -1329,7 +1329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -1337,7 +1337,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -1345,7 +1345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -1353,7 +1353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -1361,7 +1361,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -1369,7 +1369,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -1377,7 +1377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -1385,7 +1385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -1393,7 +1393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -1401,7 +1401,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -1409,7 +1409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -1417,7 +1417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -1425,7 +1425,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -1433,7 +1433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>3</v>
       </c>
@@ -1441,7 +1441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>29</v>
       </c>
@@ -1449,7 +1449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>30</v>
       </c>
@@ -1457,7 +1457,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>31</v>
       </c>
@@ -1465,7 +1465,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>32</v>
       </c>
@@ -1473,7 +1473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>33</v>
       </c>
@@ -1481,7 +1481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>34</v>
       </c>
@@ -1489,7 +1489,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>35</v>
       </c>
@@ -1497,7 +1497,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>36</v>
       </c>
@@ -1505,7 +1505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>37</v>
       </c>
@@ -1521,12 +1521,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C5D2E10-6D88-4A1E-9C1A-BD9E15FD6A9D}">
   <dimension ref="A1:B145"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>185</v>
       </c>
@@ -1534,7 +1534,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>39</v>
       </c>
@@ -1542,7 +1542,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>40</v>
       </c>
@@ -1550,7 +1550,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>41</v>
       </c>
@@ -1558,7 +1558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>42</v>
       </c>
@@ -1566,7 +1566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -1574,7 +1574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -1582,7 +1582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>45</v>
       </c>
@@ -1590,7 +1590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>46</v>
       </c>
@@ -1598,7 +1598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -1606,7 +1606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>48</v>
       </c>
@@ -1614,7 +1614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>49</v>
       </c>
@@ -1622,7 +1622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>50</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>51</v>
       </c>
@@ -1638,7 +1638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>52</v>
       </c>
@@ -1646,7 +1646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>53</v>
       </c>
@@ -1654,7 +1654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>54</v>
       </c>
@@ -1662,7 +1662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>55</v>
       </c>
@@ -1670,7 +1670,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>56</v>
       </c>
@@ -1678,7 +1678,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>57</v>
       </c>
@@ -1686,7 +1686,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>58</v>
       </c>
@@ -1694,7 +1694,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>59</v>
       </c>
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>60</v>
       </c>
@@ -1710,7 +1710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>61</v>
       </c>
@@ -1718,7 +1718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>62</v>
       </c>
@@ -1726,7 +1726,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>63</v>
       </c>
@@ -1734,7 +1734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>64</v>
       </c>
@@ -1742,7 +1742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>65</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>66</v>
       </c>
@@ -1758,7 +1758,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>67</v>
       </c>
@@ -1766,7 +1766,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>68</v>
       </c>
@@ -1774,7 +1774,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>69</v>
       </c>
@@ -1782,7 +1782,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>70</v>
       </c>
@@ -1790,7 +1790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>71</v>
       </c>
@@ -1798,7 +1798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>72</v>
       </c>
@@ -1806,7 +1806,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>73</v>
       </c>
@@ -1814,7 +1814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>74</v>
       </c>
@@ -1822,7 +1822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>75</v>
       </c>
@@ -1830,7 +1830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>76</v>
       </c>
@@ -1838,7 +1838,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>77</v>
       </c>
@@ -1846,7 +1846,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>78</v>
       </c>
@@ -1854,7 +1854,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>79</v>
       </c>
@@ -1862,7 +1862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>80</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>81</v>
       </c>
@@ -1878,7 +1878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>82</v>
       </c>
@@ -1886,7 +1886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>83</v>
       </c>
@@ -1894,7 +1894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>84</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>85</v>
       </c>
@@ -1910,7 +1910,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>86</v>
       </c>
@@ -1918,7 +1918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>87</v>
       </c>
@@ -1926,7 +1926,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>88</v>
       </c>
@@ -1934,7 +1934,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>89</v>
       </c>
@@ -1942,7 +1942,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>90</v>
       </c>
@@ -1950,7 +1950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>91</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>92</v>
       </c>
@@ -1966,7 +1966,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>93</v>
       </c>
@@ -1974,7 +1974,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>94</v>
       </c>
@@ -1982,7 +1982,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>95</v>
       </c>
@@ -1990,7 +1990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>96</v>
       </c>
@@ -1998,7 +1998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>97</v>
       </c>
@@ -2006,7 +2006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>98</v>
       </c>
@@ -2014,7 +2014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>99</v>
       </c>
@@ -2022,7 +2022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>100</v>
       </c>
@@ -2030,7 +2030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>101</v>
       </c>
@@ -2038,7 +2038,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>102</v>
       </c>
@@ -2046,7 +2046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>103</v>
       </c>
@@ -2054,7 +2054,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>104</v>
       </c>
@@ -2062,7 +2062,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>105</v>
       </c>
@@ -2070,7 +2070,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>106</v>
       </c>
@@ -2078,7 +2078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>107</v>
       </c>
@@ -2086,7 +2086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>108</v>
       </c>
@@ -2094,7 +2094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>109</v>
       </c>
@@ -2102,7 +2102,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>110</v>
       </c>
@@ -2110,7 +2110,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>111</v>
       </c>
@@ -2118,7 +2118,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>112</v>
       </c>
@@ -2126,7 +2126,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>113</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>114</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>115</v>
       </c>
@@ -2150,7 +2150,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>116</v>
       </c>
@@ -2158,7 +2158,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>117</v>
       </c>
@@ -2166,7 +2166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>118</v>
       </c>
@@ -2174,7 +2174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>119</v>
       </c>
@@ -2182,7 +2182,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>120</v>
       </c>
@@ -2190,7 +2190,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>121</v>
       </c>
@@ -2198,7 +2198,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>122</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>123</v>
       </c>
@@ -2214,7 +2214,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>124</v>
       </c>
@@ -2222,7 +2222,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>125</v>
       </c>
@@ -2230,7 +2230,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>126</v>
       </c>
@@ -2238,7 +2238,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>127</v>
       </c>
@@ -2246,7 +2246,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>128</v>
       </c>
@@ -2254,7 +2254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>129</v>
       </c>
@@ -2262,7 +2262,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>130</v>
       </c>
@@ -2270,7 +2270,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>131</v>
       </c>
@@ -2278,7 +2278,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>132</v>
       </c>
@@ -2286,7 +2286,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>133</v>
       </c>
@@ -2294,7 +2294,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>134</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>135</v>
       </c>
@@ -2310,7 +2310,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>136</v>
       </c>
@@ -2318,7 +2318,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>137</v>
       </c>
@@ -2326,7 +2326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>138</v>
       </c>
@@ -2334,7 +2334,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>139</v>
       </c>
@@ -2342,7 +2342,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>140</v>
       </c>
@@ -2350,7 +2350,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>141</v>
       </c>
@@ -2358,7 +2358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>142</v>
       </c>
@@ -2366,7 +2366,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>143</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>144</v>
       </c>
@@ -2382,7 +2382,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>145</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>146</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>147</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>148</v>
       </c>
@@ -2414,7 +2414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>149</v>
       </c>
@@ -2422,7 +2422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>150</v>
       </c>
@@ -2430,7 +2430,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>151</v>
       </c>
@@ -2438,7 +2438,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>152</v>
       </c>
@@ -2446,7 +2446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>153</v>
       </c>
@@ -2454,7 +2454,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>154</v>
       </c>
@@ -2462,7 +2462,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>155</v>
       </c>
@@ -2470,7 +2470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>156</v>
       </c>
@@ -2478,7 +2478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>157</v>
       </c>
@@ -2486,7 +2486,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>158</v>
       </c>
@@ -2494,7 +2494,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>159</v>
       </c>
@@ -2502,7 +2502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>160</v>
       </c>
@@ -2510,7 +2510,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>161</v>
       </c>
@@ -2518,7 +2518,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>162</v>
       </c>
@@ -2526,7 +2526,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>163</v>
       </c>
@@ -2534,7 +2534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>164</v>
       </c>
@@ -2542,7 +2542,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>165</v>
       </c>
@@ -2550,7 +2550,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>166</v>
       </c>
@@ -2558,7 +2558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>167</v>
       </c>
@@ -2566,7 +2566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>168</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>169</v>
       </c>
@@ -2582,7 +2582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>170</v>
       </c>
@@ -2590,7 +2590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>171</v>
       </c>
@@ -2598,7 +2598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>172</v>
       </c>
@@ -2606,7 +2606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>173</v>
       </c>
@@ -2614,7 +2614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>174</v>
       </c>
@@ -2622,7 +2622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>175</v>
       </c>
@@ -2630,7 +2630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>176</v>
       </c>
@@ -2638,7 +2638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>177</v>
       </c>
@@ -2646,7 +2646,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>178</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>179</v>
       </c>
@@ -2662,7 +2662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>180</v>
       </c>
@@ -2670,7 +2670,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>181</v>
       </c>
@@ -2678,7 +2678,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>182</v>
       </c>
@@ -2699,9 +2699,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B82051EE-CB34-4773-B6E9-985CB3357CE5}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>221</v>
       </c>
@@ -2709,7 +2709,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>222</v>
       </c>
@@ -2717,7 +2717,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>223</v>
       </c>
@@ -2725,7 +2725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>224</v>
       </c>
@@ -2733,7 +2733,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>225</v>
       </c>
@@ -2741,7 +2741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>226</v>
       </c>
@@ -2749,7 +2749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>227</v>
       </c>
@@ -2757,7 +2757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>228</v>
       </c>
@@ -2765,7 +2765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>229</v>
       </c>
@@ -2781,9 +2781,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C7942D6-5BBA-4326-BEB2-07D45E712A14}">
   <dimension ref="A1:B31"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>188</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>189</v>
       </c>
@@ -2799,7 +2799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>190</v>
       </c>
@@ -2807,7 +2807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>191</v>
       </c>
@@ -2815,7 +2815,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>192</v>
       </c>
@@ -2823,7 +2823,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>193</v>
       </c>
@@ -2831,7 +2831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>194</v>
       </c>
@@ -2839,7 +2839,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>195</v>
       </c>
@@ -2847,7 +2847,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>196</v>
       </c>
@@ -2855,7 +2855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>197</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>198</v>
       </c>
@@ -2871,7 +2871,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>199</v>
       </c>
@@ -2879,7 +2879,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>200</v>
       </c>
@@ -2887,7 +2887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>201</v>
       </c>
@@ -2895,7 +2895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>202</v>
       </c>
@@ -2903,7 +2903,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>203</v>
       </c>
@@ -2911,7 +2911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>204</v>
       </c>
@@ -2919,7 +2919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>205</v>
       </c>
@@ -2927,7 +2927,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>206</v>
       </c>
@@ -2935,7 +2935,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>207</v>
       </c>
@@ -2943,7 +2943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>208</v>
       </c>
@@ -2951,7 +2951,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>209</v>
       </c>
@@ -2959,7 +2959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>210</v>
       </c>
@@ -2967,7 +2967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>211</v>
       </c>
@@ -2975,7 +2975,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>212</v>
       </c>
@@ -2983,7 +2983,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>213</v>
       </c>
@@ -2991,7 +2991,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>208</v>
       </c>
@@ -2999,7 +2999,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>214</v>
       </c>
@@ -3007,7 +3007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>215</v>
       </c>
@@ -3015,7 +3015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>216</v>
       </c>
@@ -3023,7 +3023,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>217</v>
       </c>
@@ -3047,9 +3047,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A951553-3765-459F-BC61-BDBD26E96FE5}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>219</v>
       </c>
@@ -3057,7 +3057,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3065,7 +3065,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3073,7 +3073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3081,7 +3081,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3097,9 +3097,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{755CD133-F9DD-44F8-9E58-F17622E607C5}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>183</v>
       </c>
@@ -3107,7 +3107,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>184</v>
       </c>
@@ -3123,9 +3123,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C358E473-EC7A-41C0-8602-044D340269A5}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>259</v>
       </c>
@@ -3133,7 +3133,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>231</v>
       </c>
@@ -3141,7 +3141,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>232</v>
       </c>
@@ -3149,7 +3149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>233</v>
       </c>
@@ -3157,7 +3157,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>234</v>
       </c>
@@ -3165,7 +3165,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>235</v>
       </c>
@@ -3173,7 +3173,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>236</v>
       </c>
@@ -3181,7 +3181,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>237</v>
       </c>
@@ -3189,7 +3189,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>238</v>
       </c>
@@ -3197,7 +3197,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>239</v>
       </c>
@@ -3205,7 +3205,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>240</v>
       </c>
@@ -3213,7 +3213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>241</v>
       </c>
@@ -3221,7 +3221,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>242</v>
       </c>
@@ -3229,7 +3229,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>243</v>
       </c>
@@ -3237,7 +3237,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>244</v>
       </c>
@@ -3245,7 +3245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>245</v>
       </c>
@@ -3253,7 +3253,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>246</v>
       </c>
@@ -3261,7 +3261,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>247</v>
       </c>
@@ -3269,7 +3269,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>248</v>
       </c>
@@ -3285,9 +3285,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96D5B3E0-498C-4AB7-BB30-7BCE295E19AC}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>250</v>
       </c>
@@ -3295,7 +3295,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>197</v>
       </c>
@@ -3303,7 +3303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>251</v>
       </c>
@@ -3311,7 +3311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>252</v>
       </c>
@@ -3319,7 +3319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>253</v>
       </c>
@@ -3327,7 +3327,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>254</v>
       </c>
@@ -3335,7 +3335,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>255</v>
       </c>
@@ -3343,7 +3343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>256</v>
       </c>
@@ -3351,7 +3351,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>257</v>
       </c>
@@ -3367,9 +3367,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5D817F8-1014-4E28-A827-54661E8BA006}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>261</v>
       </c>
@@ -3378,7 +3378,7 @@
       </c>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2015</v>
       </c>
@@ -3386,7 +3386,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2018</v>
       </c>
@@ -3394,7 +3394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2019</v>
       </c>
@@ -3402,7 +3402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2020</v>
       </c>
@@ -3410,7 +3410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2025</v>
       </c>
@@ -3418,7 +3418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2030</v>
       </c>
@@ -3426,7 +3426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2035</v>
       </c>
@@ -3434,7 +3434,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2040</v>
       </c>
@@ -3442,7 +3442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2045</v>
       </c>
@@ -3450,7 +3450,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2050</v>
       </c>

</xml_diff>